<commit_message>
colorized day cells same way as Daily Status
</commit_message>
<xml_diff>
--- a/api/templates/utilization_per_instrument_day/en.xlsx
+++ b/api/templates/utilization_per_instrument_day/en.xlsx
@@ -12,22 +12,18 @@
     <workbookView xWindow="35568" yWindow="1332" windowWidth="22992" windowHeight="16080" tabRatio="815"/>
   </bookViews>
   <sheets>
-    <sheet name="Utilization" sheetId="1" r:id="rId1"/>
-    <sheet name="Detailed by assay" sheetId="5" r:id="rId2"/>
+    <sheet name="Utilization Raw Data" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="162913" fullPrecision="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
   <si>
     <t>&lt;Table&gt;</t>
   </si>
   <si>
-    <t>&lt;serial&gt;</t>
-  </si>
-  <si>
     <t>Dates: &lt;Dates&gt;</t>
   </si>
   <si>
@@ -37,52 +33,37 @@
     <t>Device</t>
   </si>
   <si>
-    <t>Serial</t>
-  </si>
-  <si>
-    <t>Last Upload</t>
-  </si>
-  <si>
     <t>LGA: &lt;Lgas&gt;</t>
   </si>
   <si>
     <t>&lt;name&gt;</t>
   </si>
   <si>
-    <t>&lt;lastUploadOn&gt;</t>
-  </si>
-  <si>
-    <t>Maintenance status</t>
-  </si>
-  <si>
-    <t>&lt;deviceApprovalStatus&gt;</t>
-  </si>
-  <si>
-    <t>&lt;deviceMaintenanceStatus&gt;</t>
-  </si>
-  <si>
-    <t>Status</t>
-  </si>
-  <si>
-    <t>Device Activity by Assay</t>
-  </si>
-  <si>
-    <t>Assay</t>
-  </si>
-  <si>
-    <t>&lt;assayName&gt;</t>
-  </si>
-  <si>
     <t>Utilization per instrument/day</t>
+  </si>
+  <si>
+    <t>Device Capacity</t>
+  </si>
+  <si>
+    <t>Total Results in period</t>
+  </si>
+  <si>
+    <t>&lt;totalResults&gt;</t>
+  </si>
+  <si>
+    <t>&lt;deviceCapacity&gt;</t>
+  </si>
+  <si>
+    <t>Utilization Rate</t>
+  </si>
+  <si>
+    <t>&lt;utilizationRate&gt;</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="[$-409]mmmm\ d\,\ yyyy;@"/>
-  </numFmts>
   <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
@@ -204,13 +185,19 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="43">
     <cellStyle name="Followed Hyperlink" xfId="2" builtinId="9" hidden="1"/>
@@ -620,203 +607,73 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="31.796875" customWidth="1"/>
-    <col min="2" max="2" width="26.296875" customWidth="1"/>
-    <col min="3" max="3" width="18.19921875" customWidth="1"/>
-    <col min="4" max="4" width="29.5" style="1" customWidth="1"/>
-    <col min="5" max="5" width="18.796875" style="1" customWidth="1"/>
+    <col min="2" max="2" width="12.796875" customWidth="1"/>
+    <col min="3" max="3" width="14.296875" customWidth="1"/>
+    <col min="4" max="4" width="14.296875" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="21" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:4" ht="21" x14ac:dyDescent="0.4">
       <c r="A1" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="1"/>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="1"/>
-      <c r="C2" s="1"/>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A3" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" s="1"/>
-      <c r="C3" s="1"/>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="B4" s="1"/>
-      <c r="C4" s="1"/>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" s="1"/>
-      <c r="B5" s="1"/>
-      <c r="C5" s="1"/>
-    </row>
-    <row r="6" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    </row>
+    <row r="6" spans="1:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B6" s="1"/>
-      <c r="C6" s="1"/>
-    </row>
-    <row r="7" spans="1:5" ht="33" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    </row>
+    <row r="7" spans="1:4" ht="33" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="B7" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A8" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="C7" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="D7" s="3" t="s">
+      <c r="B8" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C8" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="E7" s="3" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A8" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="C8" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="D8" s="5" t="s">
+      <c r="D8" s="7" t="s">
         <v>12</v>
-      </c>
-      <c r="E8" s="5" t="s">
-        <v>11</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" orientation="portrait" r:id="rId1"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F8"/>
-  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="38.796875" customWidth="1"/>
-    <col min="2" max="2" width="38.796875" style="1" customWidth="1"/>
-    <col min="3" max="3" width="37.296875" customWidth="1"/>
-    <col min="4" max="4" width="36.59765625" customWidth="1"/>
-    <col min="5" max="5" width="19.296875" customWidth="1"/>
-    <col min="6" max="6" width="17.19921875" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:6" ht="21" x14ac:dyDescent="0.4">
-      <c r="A1" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="C2" s="1"/>
-      <c r="D2" s="1"/>
-      <c r="E2" s="1"/>
-      <c r="F2" s="1"/>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A3" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="C3" s="1"/>
-      <c r="D3" s="1"/>
-      <c r="E3" s="1"/>
-      <c r="F3" s="1"/>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="C4" s="1"/>
-      <c r="D4" s="1"/>
-      <c r="E4" s="1"/>
-      <c r="F4" s="1"/>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A5" s="1"/>
-      <c r="C5" s="1"/>
-      <c r="D5" s="1"/>
-      <c r="E5" s="1"/>
-      <c r="F5" s="1"/>
-    </row>
-    <row r="6" spans="1:6" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C6" s="1"/>
-      <c r="D6" s="1"/>
-      <c r="E6" s="1"/>
-      <c r="F6" s="1"/>
-    </row>
-    <row r="7" spans="1:6" ht="33" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="E7" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="F7" s="3" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A8" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="C8" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="D8" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="E8" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="F8" s="5" t="s">
-        <v>11</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
formating template Excel file
</commit_message>
<xml_diff>
--- a/api/templates/utilization_per_instrument_day/en.xlsx
+++ b/api/templates/utilization_per_instrument_day/en.xlsx
@@ -194,10 +194,10 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="43">
     <cellStyle name="Followed Hyperlink" xfId="2" builtinId="9" hidden="1"/>
@@ -612,8 +612,8 @@
   <cols>
     <col min="1" max="1" width="31.796875" customWidth="1"/>
     <col min="2" max="2" width="12.796875" customWidth="1"/>
-    <col min="3" max="3" width="14.296875" customWidth="1"/>
-    <col min="4" max="4" width="14.296875" style="1" customWidth="1"/>
+    <col min="3" max="3" width="10.59765625" customWidth="1"/>
+    <col min="4" max="4" width="10.3984375" style="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="21" x14ac:dyDescent="0.4">
@@ -651,10 +651,10 @@
       <c r="B7" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="C7" s="6" t="s">
+      <c r="C7" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="D7" s="6" t="s">
+      <c r="D7" s="7" t="s">
         <v>11</v>
       </c>
     </row>
@@ -668,7 +668,7 @@
       <c r="C8" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="D8" s="7" t="s">
+      <c r="D8" s="6" t="s">
         <v>12</v>
       </c>
     </row>

</xml_diff>